<commit_message>
Remove Dealio.pro/SendFuse names from all client-facing surfaces; formalize comps PDF preservation workflow
</commit_message>
<xml_diff>
--- a/product-templates/Newtree_Internal_Working_Files_Template.xlsx
+++ b/product-templates/Newtree_Internal_Working_Files_Template.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -517,7 +517,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr"/>
     </row>
@@ -610,7 +609,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -714,7 +712,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Dealio.pro Comps Report, subject property block</t>
+          <t>Comps_Report_[Property Address].pdf, subject property block</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -1104,7 +1102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1118,6 +1116,7 @@
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1190,6 +1189,11 @@
           <t>Reasoning Notes</t>
         </is>
       </c>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Source PDF (saved filename)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -1245,6 +1249,11 @@
       <c r="K5" s="6" t="inlineStr">
         <is>
           <t>EXAMPLE ROW -- verified transaction pair on same property (Rule 1); individual buyer + FHA financing + detailed renovation description; $137/sqft.</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Comps_Report_16120_Harvard_Ave.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>